<commit_message>
Repair and validate scripted Excel calibration workbooks
Generate real handle references, exclude settings headers from factory input, separate route and knot data, and reserve explicit report array ranges so the examples recalculate without manual repair.

Add portable workbook contracts to CI, an isolated native Excel runner with quote perturbation checks, and consolidated review and performance evidence.
</commit_message>
<xml_diff>
--- a/dal-excel/examples/012.interpolate_curve_script.xlsx
+++ b/dal-excel/examples/012.interpolate_curve_script.xlsx
@@ -20,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="0.000E+00"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -91,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -100,6 +101,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -497,7 +510,7 @@
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="17" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
-    <col width="91" customWidth="1" min="27" max="27"/>
+    <col width="60" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -956,7 +969,7 @@
         </is>
       </c>
       <c r="AA21" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$21:$C$25,$E$21:$F$31,$H$21:$P$23,$S$21:$Y$23,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$21:$C$25,$E$22:$F$31,$H$21:$P$23,$S$21:$Y$23,)</f>
         <v/>
       </c>
     </row>
@@ -1407,7 +1420,7 @@
         </is>
       </c>
       <c r="AA36" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$36:$C$40,$E$36:$F$46,$H$36:$P$38,$S$36:$Y$38,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$36:$C$40,$E$37:$F$46,$H$36:$P$38,$S$36:$Y$38,)</f>
         <v/>
       </c>
     </row>
@@ -1858,7 +1871,7 @@
         </is>
       </c>
       <c r="AA51" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$51:$C$55,$E$51:$F$61,$H$51:$P$53,$S$51:$Y$53,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$51:$C$55,$E$52:$F$61,$H$51:$P$53,$S$51:$Y$53,)</f>
         <v/>
       </c>
     </row>
@@ -2309,7 +2322,7 @@
         </is>
       </c>
       <c r="AA66" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$66:$C$70,$E$66:$F$76,$H$66:$P$68,$S$66:$Y$68,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$66:$C$70,$E$67:$F$76,$H$66:$P$68,$S$66:$Y$68,)</f>
         <v/>
       </c>
     </row>
@@ -2760,7 +2773,7 @@
         </is>
       </c>
       <c r="AA81" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$81:$C$85,$E$81:$F$91,$H$81:$P$83,$S$81:$Y$83,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$81:$C$85,$E$82:$F$91,$H$81:$P$83,$S$81:$Y$83,)</f>
         <v/>
       </c>
     </row>
@@ -3211,7 +3224,7 @@
         </is>
       </c>
       <c r="AA96" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$96:$C$100,$E$96:$F$106,$H$96:$P$98,$S$96:$Y$98,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$96:$C$100,$E$97:$F$106,$H$96:$P$98,$S$96:$Y$98,)</f>
         <v/>
       </c>
     </row>
@@ -3662,7 +3675,7 @@
         </is>
       </c>
       <c r="AA111" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$111:$C$115,$E$111:$F$121,$H$111:$P$113,$S$111:$Y$113,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$111:$C$115,$E$112:$F$121,$H$111:$P$113,$S$111:$Y$113,)</f>
         <v/>
       </c>
     </row>
@@ -4113,7 +4126,7 @@
         </is>
       </c>
       <c r="AA126" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$126:$C$130,$E$126:$F$136,$H$126:$P$128,$S$126:$Y$128,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$126:$C$130,$E$127:$F$136,$H$126:$P$128,$S$126:$Y$128,)</f>
         <v/>
       </c>
     </row>
@@ -4564,7 +4577,7 @@
         </is>
       </c>
       <c r="AA141" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$141:$C$145,$E$141:$F$151,$H$141:$P$143,$S$141:$Y$143,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$141:$C$145,$E$142:$F$151,$H$141:$P$143,$S$141:$Y$143,)</f>
         <v/>
       </c>
     </row>
@@ -5015,7 +5028,7 @@
         </is>
       </c>
       <c r="AA156" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$156:$C$164,$E$156:$F$166,$H$156:$P$158,$S$156:$Y$158,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$156:$C$164,$E$157:$F$166,$H$156:$P$158,$S$156:$Y$158,)</f>
         <v/>
       </c>
     </row>
@@ -5526,7 +5539,7 @@
         </is>
       </c>
       <c r="AA171" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$171:$C$183,$E$171:$F$181,$H$171:$P$173,$S$171:$Y$173,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$171:$C$183,$E$172:$F$181,$H$171:$P$173,$S$171:$Y$173,)</f>
         <v/>
       </c>
     </row>
@@ -6101,7 +6114,7 @@
         </is>
       </c>
       <c r="AA188" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$188:$C$204,$E$188:$F$198,$H$188:$P$190,$S$188:$Y$190,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$188:$C$204,$E$189:$F$198,$H$188:$P$190,$S$188:$Y$190,)</f>
         <v/>
       </c>
     </row>
@@ -6744,7 +6757,7 @@
         </is>
       </c>
       <c r="AA209" s="4">
-        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$209:$C$231,$E$209:$F$219,$H$209:$P$211,$S$209:$Y$211,)</f>
+        <f>SCRIPTINSTRUMENTDEFINITION.NEW($A$209:$C$231,$E$210:$F$219,$H$209:$P$211,$S$209:$Y$211,)</f>
         <v/>
       </c>
     </row>
@@ -7378,17 +7391,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:V86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="67" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7413,7 +7440,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>CALIBRATIONDATES.NEW($H$5:$H$18)</f>
+        <f>CALIBRATIONDATES.NEW($L$5:$L$18)</f>
         <v/>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -7426,12 +7453,12 @@
           <t>value</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>knot_date</t>
         </is>
@@ -7444,7 +7471,7 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>CURVEINSTRUMENTGEOMETRY.NEW($D$4:$E$14)</f>
+        <f>CURVEINSTRUMENTGEOMETRY.NEW($D$5:$E$14)</f>
         <v/>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -7455,10 +7482,10 @@
       <c r="E5" s="7" t="n">
         <v>44562</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="L5" s="7" t="n">
         <v>44562</v>
       </c>
     </row>
@@ -7482,10 +7509,10 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="K6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="L6" s="7" t="n">
         <v>44635</v>
       </c>
     </row>
@@ -7496,7 +7523,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>CURVEINSTRUMENTMARKET.NEW($D$21:$E$22)</f>
+        <f>CURVEINSTRUMENTMARKET.NEW($D$22:$E$22)</f>
         <v/>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -7509,10 +7536,10 @@
           <t>ptirds</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="K7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="L7" s="7" t="n">
         <v>44727</v>
       </c>
     </row>
@@ -7531,15 +7558,14 @@
           <t>knot_dates</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>$B$4</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="n">
+      <c r="E8" s="6">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="K8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="L8" s="7" t="n">
         <v>44825</v>
       </c>
     </row>
@@ -7550,7 +7576,7 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <f>SCRIPTVALUATIONSETTINGS.NEW("ptirds-valuation",$D$25:$E$26,$B$8)</f>
+        <f>SCRIPTVALUATIONSETTINGS.NEW("ptirds-valuation",$D$26:$E$26,$B$8)</f>
         <v/>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -7563,10 +7589,10 @@
           <t>LOG_DISCOUNT</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="K9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="L9" s="7" t="n">
         <v>44916</v>
       </c>
     </row>
@@ -7577,7 +7603,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>CURVEINSTRUMENTSOLVER.NEW($D$29:$E$35)</f>
+        <f>CURVEINSTRUMENTSOLVER.NEW($D$30:$E$35)</f>
         <v/>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -7590,10 +7616,10 @@
           <t>INPUT</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="K10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="L10" s="7" t="n">
         <v>45000</v>
       </c>
     </row>
@@ -7604,7 +7630,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>CURVEINSTRUMENTCALIBRATIONOPTIONS.NEW($D$38:$E$42)</f>
+        <f>CURVEINSTRUMENTCALIBRATIONOPTIONS.NEW($D$39:$E$42)</f>
         <v/>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -7617,10 +7643,10 @@
           <t>LOG_LINEAR</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="L11" s="7" t="n">
         <v>45098</v>
       </c>
     </row>
@@ -7642,10 +7668,10 @@
       <c r="E12" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="K12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="L12" s="7" t="n">
         <v>45189</v>
       </c>
     </row>
@@ -7656,7 +7682,7 @@
         </is>
       </c>
       <c r="B13" s="4">
-        <f>CURVEINSTRUMENTCALIBRATIONSPEC.NEW($D$45:$E$50)</f>
+        <f>CURVEINSTRUMENTCALIBRATIONSPEC.NEW($D$46:$E$50)</f>
         <v/>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -7669,10 +7695,10 @@
           <t>OIS</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="K13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="L13" s="7" t="n">
         <v>45280</v>
       </c>
     </row>
@@ -7696,10 +7722,10 @@
           <t>ACT_365F</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="K14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="L14" s="7" t="n">
         <v>45366</v>
       </c>
     </row>
@@ -7713,10 +7739,10 @@
         <f>CALIBRATIONOUTCOME.GET.STATUS($B$14)</f>
         <v/>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="K15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="L15" s="7" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -7730,10 +7756,10 @@
         <f>CALIBRATIONOUTCOME.GET.REPORT($B$14)</f>
         <v/>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="K16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="L16" s="7" t="n">
         <v>46388</v>
       </c>
     </row>
@@ -7767,7 +7793,10 @@
           <t>tenor</t>
         </is>
       </c>
-      <c r="H17" s="7" t="n">
+      <c r="K17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L17" s="7" t="n">
         <v>47119</v>
       </c>
     </row>
@@ -7785,10 +7814,11 @@
           <t>OIS</t>
         </is>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="6" t="n"/>
+      <c r="K18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="L18" s="7" t="n">
         <v>48214</v>
       </c>
     </row>
@@ -7807,28 +7837,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Observation report</t>
-        </is>
-      </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
           <t>routes</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>$B$6</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4">
-        <f>CALIBRATIONREPORT.GET.OBSERVATIONS($B$16)</f>
-        <v/>
-      </c>
-    </row>
+      <c r="E22" s="6">
+        <f>$B$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24"/>
     <row r="25">
       <c r="D25" s="2" t="inlineStr">
@@ -7955,11 +7974,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>Fitted parameters</t>
-        </is>
-      </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
           <t>jacobian_mode</t>
@@ -7972,10 +7986,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4">
-        <f>CALIBRATIONREPORT.GET.PARAMETERS($B$16)</f>
-        <v/>
-      </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
           <t>difference_step</t>
@@ -8015,10 +8025,9 @@
           <t>geometry</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>$B$5</t>
-        </is>
+      <c r="E46" s="6">
+        <f>$B$5</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -8027,10 +8036,9 @@
           <t>market</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>$B$7</t>
-        </is>
+      <c r="E47" s="6">
+        <f>$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -8039,10 +8047,9 @@
           <t>valuation</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>$B$9</t>
-        </is>
+      <c r="E48" s="6">
+        <f>$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -8051,10 +8058,9 @@
           <t>observations</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>$B$12</t>
-        </is>
+      <c r="E49" s="6">
+        <f>$B$12</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -8063,11 +8069,526 @@
           <t>solver</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>$B$10</t>
-        </is>
-      </c>
+      <c r="E50" s="6">
+        <f>$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>Observation report</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="8">
+        <f t="array" ref="A55:V68">CALIBRATIONREPORT.GET.OBSERVATIONS($B$16)</f>
+        <v/>
+      </c>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8" t="n"/>
+      <c r="K55" s="8" t="n"/>
+      <c r="L55" s="9" t="n"/>
+      <c r="M55" s="8" t="n"/>
+      <c r="N55" s="9" t="n"/>
+      <c r="O55" s="9" t="n"/>
+      <c r="P55" s="8" t="n"/>
+      <c r="Q55" s="8" t="n"/>
+      <c r="R55" s="8" t="n"/>
+      <c r="S55" s="8" t="n"/>
+      <c r="T55" s="8" t="n"/>
+      <c r="U55" s="8" t="n"/>
+      <c r="V55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n"/>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="10" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="10" t="n"/>
+      <c r="I56" s="10" t="n"/>
+      <c r="J56" s="10" t="n"/>
+      <c r="K56" s="10" t="n"/>
+      <c r="L56" s="11" t="n"/>
+      <c r="M56" s="10" t="n"/>
+      <c r="N56" s="11" t="n"/>
+      <c r="O56" s="11" t="n"/>
+      <c r="P56" s="10" t="n"/>
+      <c r="Q56" s="10" t="n"/>
+      <c r="R56" s="10" t="n"/>
+      <c r="S56" s="10" t="n"/>
+      <c r="T56" s="10" t="n"/>
+      <c r="U56" s="10" t="n"/>
+      <c r="V56" s="10" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="n"/>
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="10" t="n"/>
+      <c r="D57" s="10" t="n"/>
+      <c r="E57" s="10" t="n"/>
+      <c r="F57" s="10" t="n"/>
+      <c r="G57" s="10" t="n"/>
+      <c r="H57" s="10" t="n"/>
+      <c r="I57" s="10" t="n"/>
+      <c r="J57" s="10" t="n"/>
+      <c r="K57" s="10" t="n"/>
+      <c r="L57" s="11" t="n"/>
+      <c r="M57" s="10" t="n"/>
+      <c r="N57" s="11" t="n"/>
+      <c r="O57" s="11" t="n"/>
+      <c r="P57" s="10" t="n"/>
+      <c r="Q57" s="10" t="n"/>
+      <c r="R57" s="10" t="n"/>
+      <c r="S57" s="10" t="n"/>
+      <c r="T57" s="10" t="n"/>
+      <c r="U57" s="10" t="n"/>
+      <c r="V57" s="10" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n"/>
+      <c r="B58" s="10" t="n"/>
+      <c r="C58" s="10" t="n"/>
+      <c r="D58" s="10" t="n"/>
+      <c r="E58" s="10" t="n"/>
+      <c r="F58" s="10" t="n"/>
+      <c r="G58" s="10" t="n"/>
+      <c r="H58" s="10" t="n"/>
+      <c r="I58" s="10" t="n"/>
+      <c r="J58" s="10" t="n"/>
+      <c r="K58" s="10" t="n"/>
+      <c r="L58" s="11" t="n"/>
+      <c r="M58" s="10" t="n"/>
+      <c r="N58" s="11" t="n"/>
+      <c r="O58" s="11" t="n"/>
+      <c r="P58" s="10" t="n"/>
+      <c r="Q58" s="10" t="n"/>
+      <c r="R58" s="10" t="n"/>
+      <c r="S58" s="10" t="n"/>
+      <c r="T58" s="10" t="n"/>
+      <c r="U58" s="10" t="n"/>
+      <c r="V58" s="10" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="n"/>
+      <c r="B59" s="10" t="n"/>
+      <c r="C59" s="10" t="n"/>
+      <c r="D59" s="10" t="n"/>
+      <c r="E59" s="10" t="n"/>
+      <c r="F59" s="10" t="n"/>
+      <c r="G59" s="10" t="n"/>
+      <c r="H59" s="10" t="n"/>
+      <c r="I59" s="10" t="n"/>
+      <c r="J59" s="10" t="n"/>
+      <c r="K59" s="10" t="n"/>
+      <c r="L59" s="11" t="n"/>
+      <c r="M59" s="10" t="n"/>
+      <c r="N59" s="11" t="n"/>
+      <c r="O59" s="11" t="n"/>
+      <c r="P59" s="10" t="n"/>
+      <c r="Q59" s="10" t="n"/>
+      <c r="R59" s="10" t="n"/>
+      <c r="S59" s="10" t="n"/>
+      <c r="T59" s="10" t="n"/>
+      <c r="U59" s="10" t="n"/>
+      <c r="V59" s="10" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="n"/>
+      <c r="B60" s="10" t="n"/>
+      <c r="C60" s="10" t="n"/>
+      <c r="D60" s="10" t="n"/>
+      <c r="E60" s="10" t="n"/>
+      <c r="F60" s="10" t="n"/>
+      <c r="G60" s="10" t="n"/>
+      <c r="H60" s="10" t="n"/>
+      <c r="I60" s="10" t="n"/>
+      <c r="J60" s="10" t="n"/>
+      <c r="K60" s="10" t="n"/>
+      <c r="L60" s="11" t="n"/>
+      <c r="M60" s="10" t="n"/>
+      <c r="N60" s="11" t="n"/>
+      <c r="O60" s="11" t="n"/>
+      <c r="P60" s="10" t="n"/>
+      <c r="Q60" s="10" t="n"/>
+      <c r="R60" s="10" t="n"/>
+      <c r="S60" s="10" t="n"/>
+      <c r="T60" s="10" t="n"/>
+      <c r="U60" s="10" t="n"/>
+      <c r="V60" s="10" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="n"/>
+      <c r="B61" s="10" t="n"/>
+      <c r="C61" s="10" t="n"/>
+      <c r="D61" s="10" t="n"/>
+      <c r="E61" s="10" t="n"/>
+      <c r="F61" s="10" t="n"/>
+      <c r="G61" s="10" t="n"/>
+      <c r="H61" s="10" t="n"/>
+      <c r="I61" s="10" t="n"/>
+      <c r="J61" s="10" t="n"/>
+      <c r="K61" s="10" t="n"/>
+      <c r="L61" s="11" t="n"/>
+      <c r="M61" s="10" t="n"/>
+      <c r="N61" s="11" t="n"/>
+      <c r="O61" s="11" t="n"/>
+      <c r="P61" s="10" t="n"/>
+      <c r="Q61" s="10" t="n"/>
+      <c r="R61" s="10" t="n"/>
+      <c r="S61" s="10" t="n"/>
+      <c r="T61" s="10" t="n"/>
+      <c r="U61" s="10" t="n"/>
+      <c r="V61" s="10" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="n"/>
+      <c r="B62" s="10" t="n"/>
+      <c r="C62" s="10" t="n"/>
+      <c r="D62" s="10" t="n"/>
+      <c r="E62" s="10" t="n"/>
+      <c r="F62" s="10" t="n"/>
+      <c r="G62" s="10" t="n"/>
+      <c r="H62" s="10" t="n"/>
+      <c r="I62" s="10" t="n"/>
+      <c r="J62" s="10" t="n"/>
+      <c r="K62" s="10" t="n"/>
+      <c r="L62" s="11" t="n"/>
+      <c r="M62" s="10" t="n"/>
+      <c r="N62" s="11" t="n"/>
+      <c r="O62" s="11" t="n"/>
+      <c r="P62" s="10" t="n"/>
+      <c r="Q62" s="10" t="n"/>
+      <c r="R62" s="10" t="n"/>
+      <c r="S62" s="10" t="n"/>
+      <c r="T62" s="10" t="n"/>
+      <c r="U62" s="10" t="n"/>
+      <c r="V62" s="10" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="n"/>
+      <c r="B63" s="10" t="n"/>
+      <c r="C63" s="10" t="n"/>
+      <c r="D63" s="10" t="n"/>
+      <c r="E63" s="10" t="n"/>
+      <c r="F63" s="10" t="n"/>
+      <c r="G63" s="10" t="n"/>
+      <c r="H63" s="10" t="n"/>
+      <c r="I63" s="10" t="n"/>
+      <c r="J63" s="10" t="n"/>
+      <c r="K63" s="10" t="n"/>
+      <c r="L63" s="11" t="n"/>
+      <c r="M63" s="10" t="n"/>
+      <c r="N63" s="11" t="n"/>
+      <c r="O63" s="11" t="n"/>
+      <c r="P63" s="10" t="n"/>
+      <c r="Q63" s="10" t="n"/>
+      <c r="R63" s="10" t="n"/>
+      <c r="S63" s="10" t="n"/>
+      <c r="T63" s="10" t="n"/>
+      <c r="U63" s="10" t="n"/>
+      <c r="V63" s="10" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="n"/>
+      <c r="B64" s="10" t="n"/>
+      <c r="C64" s="10" t="n"/>
+      <c r="D64" s="10" t="n"/>
+      <c r="E64" s="10" t="n"/>
+      <c r="F64" s="10" t="n"/>
+      <c r="G64" s="10" t="n"/>
+      <c r="H64" s="10" t="n"/>
+      <c r="I64" s="10" t="n"/>
+      <c r="J64" s="10" t="n"/>
+      <c r="K64" s="10" t="n"/>
+      <c r="L64" s="11" t="n"/>
+      <c r="M64" s="10" t="n"/>
+      <c r="N64" s="11" t="n"/>
+      <c r="O64" s="11" t="n"/>
+      <c r="P64" s="10" t="n"/>
+      <c r="Q64" s="10" t="n"/>
+      <c r="R64" s="10" t="n"/>
+      <c r="S64" s="10" t="n"/>
+      <c r="T64" s="10" t="n"/>
+      <c r="U64" s="10" t="n"/>
+      <c r="V64" s="10" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="n"/>
+      <c r="B65" s="10" t="n"/>
+      <c r="C65" s="10" t="n"/>
+      <c r="D65" s="10" t="n"/>
+      <c r="E65" s="10" t="n"/>
+      <c r="F65" s="10" t="n"/>
+      <c r="G65" s="10" t="n"/>
+      <c r="H65" s="10" t="n"/>
+      <c r="I65" s="10" t="n"/>
+      <c r="J65" s="10" t="n"/>
+      <c r="K65" s="10" t="n"/>
+      <c r="L65" s="11" t="n"/>
+      <c r="M65" s="10" t="n"/>
+      <c r="N65" s="11" t="n"/>
+      <c r="O65" s="11" t="n"/>
+      <c r="P65" s="10" t="n"/>
+      <c r="Q65" s="10" t="n"/>
+      <c r="R65" s="10" t="n"/>
+      <c r="S65" s="10" t="n"/>
+      <c r="T65" s="10" t="n"/>
+      <c r="U65" s="10" t="n"/>
+      <c r="V65" s="10" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="n"/>
+      <c r="B66" s="10" t="n"/>
+      <c r="C66" s="10" t="n"/>
+      <c r="D66" s="10" t="n"/>
+      <c r="E66" s="10" t="n"/>
+      <c r="F66" s="10" t="n"/>
+      <c r="G66" s="10" t="n"/>
+      <c r="H66" s="10" t="n"/>
+      <c r="I66" s="10" t="n"/>
+      <c r="J66" s="10" t="n"/>
+      <c r="K66" s="10" t="n"/>
+      <c r="L66" s="11" t="n"/>
+      <c r="M66" s="10" t="n"/>
+      <c r="N66" s="11" t="n"/>
+      <c r="O66" s="11" t="n"/>
+      <c r="P66" s="10" t="n"/>
+      <c r="Q66" s="10" t="n"/>
+      <c r="R66" s="10" t="n"/>
+      <c r="S66" s="10" t="n"/>
+      <c r="T66" s="10" t="n"/>
+      <c r="U66" s="10" t="n"/>
+      <c r="V66" s="10" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="n"/>
+      <c r="B67" s="10" t="n"/>
+      <c r="C67" s="10" t="n"/>
+      <c r="D67" s="10" t="n"/>
+      <c r="E67" s="10" t="n"/>
+      <c r="F67" s="10" t="n"/>
+      <c r="G67" s="10" t="n"/>
+      <c r="H67" s="10" t="n"/>
+      <c r="I67" s="10" t="n"/>
+      <c r="J67" s="10" t="n"/>
+      <c r="K67" s="10" t="n"/>
+      <c r="L67" s="11" t="n"/>
+      <c r="M67" s="10" t="n"/>
+      <c r="N67" s="11" t="n"/>
+      <c r="O67" s="11" t="n"/>
+      <c r="P67" s="10" t="n"/>
+      <c r="Q67" s="10" t="n"/>
+      <c r="R67" s="10" t="n"/>
+      <c r="S67" s="10" t="n"/>
+      <c r="T67" s="10" t="n"/>
+      <c r="U67" s="10" t="n"/>
+      <c r="V67" s="10" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="n"/>
+      <c r="B68" s="10" t="n"/>
+      <c r="C68" s="10" t="n"/>
+      <c r="D68" s="10" t="n"/>
+      <c r="E68" s="10" t="n"/>
+      <c r="F68" s="10" t="n"/>
+      <c r="G68" s="10" t="n"/>
+      <c r="H68" s="10" t="n"/>
+      <c r="I68" s="10" t="n"/>
+      <c r="J68" s="10" t="n"/>
+      <c r="K68" s="10" t="n"/>
+      <c r="L68" s="11" t="n"/>
+      <c r="M68" s="10" t="n"/>
+      <c r="N68" s="11" t="n"/>
+      <c r="O68" s="11" t="n"/>
+      <c r="P68" s="10" t="n"/>
+      <c r="Q68" s="10" t="n"/>
+      <c r="R68" s="10" t="n"/>
+      <c r="S68" s="10" t="n"/>
+      <c r="T68" s="10" t="n"/>
+      <c r="U68" s="10" t="n"/>
+      <c r="V68" s="10" t="n"/>
+    </row>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>Fitted parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="32" customHeight="1">
+      <c r="A73" s="8">
+        <f t="array" ref="A73:I86">CALIBRATIONREPORT.GET.PARAMETERS($B$16)</f>
+        <v/>
+      </c>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="8" t="n"/>
+      <c r="D73" s="8" t="n"/>
+      <c r="E73" s="8" t="n"/>
+      <c r="F73" s="8" t="n"/>
+      <c r="G73" s="8" t="n"/>
+      <c r="H73" s="8" t="n"/>
+      <c r="I73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="n"/>
+      <c r="B74" s="10" t="n"/>
+      <c r="C74" s="10" t="n"/>
+      <c r="D74" s="10" t="n"/>
+      <c r="E74" s="10" t="n"/>
+      <c r="F74" s="10" t="n"/>
+      <c r="G74" s="10" t="n"/>
+      <c r="H74" s="10" t="n"/>
+      <c r="I74" s="10" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="n"/>
+      <c r="B75" s="10" t="n"/>
+      <c r="C75" s="10" t="n"/>
+      <c r="D75" s="10" t="n"/>
+      <c r="E75" s="10" t="n"/>
+      <c r="F75" s="10" t="n"/>
+      <c r="G75" s="10" t="n"/>
+      <c r="H75" s="10" t="n"/>
+      <c r="I75" s="10" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="n"/>
+      <c r="B76" s="10" t="n"/>
+      <c r="C76" s="10" t="n"/>
+      <c r="D76" s="10" t="n"/>
+      <c r="E76" s="10" t="n"/>
+      <c r="F76" s="10" t="n"/>
+      <c r="G76" s="10" t="n"/>
+      <c r="H76" s="10" t="n"/>
+      <c r="I76" s="10" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="n"/>
+      <c r="B77" s="10" t="n"/>
+      <c r="C77" s="10" t="n"/>
+      <c r="D77" s="10" t="n"/>
+      <c r="E77" s="10" t="n"/>
+      <c r="F77" s="10" t="n"/>
+      <c r="G77" s="10" t="n"/>
+      <c r="H77" s="10" t="n"/>
+      <c r="I77" s="10" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="n"/>
+      <c r="B78" s="10" t="n"/>
+      <c r="C78" s="10" t="n"/>
+      <c r="D78" s="10" t="n"/>
+      <c r="E78" s="10" t="n"/>
+      <c r="F78" s="10" t="n"/>
+      <c r="G78" s="10" t="n"/>
+      <c r="H78" s="10" t="n"/>
+      <c r="I78" s="10" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="n"/>
+      <c r="B79" s="10" t="n"/>
+      <c r="C79" s="10" t="n"/>
+      <c r="D79" s="10" t="n"/>
+      <c r="E79" s="10" t="n"/>
+      <c r="F79" s="10" t="n"/>
+      <c r="G79" s="10" t="n"/>
+      <c r="H79" s="10" t="n"/>
+      <c r="I79" s="10" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="n"/>
+      <c r="B80" s="10" t="n"/>
+      <c r="C80" s="10" t="n"/>
+      <c r="D80" s="10" t="n"/>
+      <c r="E80" s="10" t="n"/>
+      <c r="F80" s="10" t="n"/>
+      <c r="G80" s="10" t="n"/>
+      <c r="H80" s="10" t="n"/>
+      <c r="I80" s="10" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="n"/>
+      <c r="B81" s="10" t="n"/>
+      <c r="C81" s="10" t="n"/>
+      <c r="D81" s="10" t="n"/>
+      <c r="E81" s="10" t="n"/>
+      <c r="F81" s="10" t="n"/>
+      <c r="G81" s="10" t="n"/>
+      <c r="H81" s="10" t="n"/>
+      <c r="I81" s="10" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="n"/>
+      <c r="B82" s="10" t="n"/>
+      <c r="C82" s="10" t="n"/>
+      <c r="D82" s="10" t="n"/>
+      <c r="E82" s="10" t="n"/>
+      <c r="F82" s="10" t="n"/>
+      <c r="G82" s="10" t="n"/>
+      <c r="H82" s="10" t="n"/>
+      <c r="I82" s="10" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="n"/>
+      <c r="B83" s="10" t="n"/>
+      <c r="C83" s="10" t="n"/>
+      <c r="D83" s="10" t="n"/>
+      <c r="E83" s="10" t="n"/>
+      <c r="F83" s="10" t="n"/>
+      <c r="G83" s="10" t="n"/>
+      <c r="H83" s="10" t="n"/>
+      <c r="I83" s="10" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="n"/>
+      <c r="B84" s="10" t="n"/>
+      <c r="C84" s="10" t="n"/>
+      <c r="D84" s="10" t="n"/>
+      <c r="E84" s="10" t="n"/>
+      <c r="F84" s="10" t="n"/>
+      <c r="G84" s="10" t="n"/>
+      <c r="H84" s="10" t="n"/>
+      <c r="I84" s="10" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="n"/>
+      <c r="B85" s="10" t="n"/>
+      <c r="C85" s="10" t="n"/>
+      <c r="D85" s="10" t="n"/>
+      <c r="E85" s="10" t="n"/>
+      <c r="F85" s="10" t="n"/>
+      <c r="G85" s="10" t="n"/>
+      <c r="H85" s="10" t="n"/>
+      <c r="I85" s="10" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="n"/>
+      <c r="B86" s="10" t="n"/>
+      <c r="C86" s="10" t="n"/>
+      <c r="D86" s="10" t="n"/>
+      <c r="E86" s="10" t="n"/>
+      <c r="F86" s="10" t="n"/>
+      <c r="G86" s="10" t="n"/>
+      <c r="H86" s="10" t="n"/>
+      <c r="I86" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8080,17 +8601,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:V86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="67" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8115,7 +8650,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>CALIBRATIONDATES.NEW($H$5:$H$18)</f>
+        <f>CALIBRATIONDATES.NEW($L$5:$L$18)</f>
         <v/>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -8128,12 +8663,12 @@
           <t>value</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>knot_date</t>
         </is>
@@ -8146,7 +8681,7 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>CURVEINSTRUMENTGEOMETRY.NEW($D$4:$E$14)</f>
+        <f>CURVEINSTRUMENTGEOMETRY.NEW($D$5:$E$14)</f>
         <v/>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -8157,10 +8692,10 @@
       <c r="E5" s="7" t="n">
         <v>44562</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="L5" s="7" t="n">
         <v>44562</v>
       </c>
     </row>
@@ -8184,10 +8719,10 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="K6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="L6" s="7" t="n">
         <v>44635</v>
       </c>
     </row>
@@ -8198,7 +8733,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>CURVEINSTRUMENTMARKET.NEW($D$21:$E$22)</f>
+        <f>CURVEINSTRUMENTMARKET.NEW($D$22:$E$22)</f>
         <v/>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -8211,10 +8746,10 @@
           <t>ptirds</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="K7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="L7" s="7" t="n">
         <v>44727</v>
       </c>
     </row>
@@ -8233,15 +8768,14 @@
           <t>knot_dates</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>$B$4</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="n">
+      <c r="E8" s="6">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="K8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="L8" s="7" t="n">
         <v>44825</v>
       </c>
     </row>
@@ -8252,7 +8786,7 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <f>SCRIPTVALUATIONSETTINGS.NEW("ptirds-valuation",$D$25:$E$26,$B$8)</f>
+        <f>SCRIPTVALUATIONSETTINGS.NEW("ptirds-valuation",$D$26:$E$26,$B$8)</f>
         <v/>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -8265,10 +8799,10 @@
           <t>LOG_DISCOUNT</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="K9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="L9" s="7" t="n">
         <v>44916</v>
       </c>
     </row>
@@ -8279,7 +8813,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>CURVEINSTRUMENTSOLVER.NEW($D$29:$E$35)</f>
+        <f>CURVEINSTRUMENTSOLVER.NEW($D$30:$E$35)</f>
         <v/>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -8292,10 +8826,10 @@
           <t>INPUT</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="K10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="L10" s="7" t="n">
         <v>45000</v>
       </c>
     </row>
@@ -8306,7 +8840,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>CURVEINSTRUMENTCALIBRATIONOPTIONS.NEW($D$38:$E$42)</f>
+        <f>CURVEINSTRUMENTCALIBRATIONOPTIONS.NEW($D$39:$E$42)</f>
         <v/>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -8319,10 +8853,10 @@
           <t>LOG_CUBIC_NATURAL</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="L11" s="7" t="n">
         <v>45098</v>
       </c>
     </row>
@@ -8344,10 +8878,10 @@
       <c r="E12" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="K12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="L12" s="7" t="n">
         <v>45189</v>
       </c>
     </row>
@@ -8358,7 +8892,7 @@
         </is>
       </c>
       <c r="B13" s="4">
-        <f>CURVEINSTRUMENTCALIBRATIONSPEC.NEW($D$45:$E$50)</f>
+        <f>CURVEINSTRUMENTCALIBRATIONSPEC.NEW($D$46:$E$50)</f>
         <v/>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -8371,10 +8905,10 @@
           <t>OIS</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="K13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="L13" s="7" t="n">
         <v>45280</v>
       </c>
     </row>
@@ -8398,10 +8932,10 @@
           <t>ACT_365F</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="K14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="L14" s="7" t="n">
         <v>45366</v>
       </c>
     </row>
@@ -8415,10 +8949,10 @@
         <f>CALIBRATIONOUTCOME.GET.STATUS($B$14)</f>
         <v/>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="K15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="L15" s="7" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -8432,10 +8966,10 @@
         <f>CALIBRATIONOUTCOME.GET.REPORT($B$14)</f>
         <v/>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="K16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="L16" s="7" t="n">
         <v>46388</v>
       </c>
     </row>
@@ -8469,7 +9003,10 @@
           <t>tenor</t>
         </is>
       </c>
-      <c r="H17" s="7" t="n">
+      <c r="K17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L17" s="7" t="n">
         <v>47119</v>
       </c>
     </row>
@@ -8487,10 +9024,11 @@
           <t>OIS</t>
         </is>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="6" t="n"/>
+      <c r="K18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="L18" s="7" t="n">
         <v>48214</v>
       </c>
     </row>
@@ -8509,28 +9047,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Observation report</t>
-        </is>
-      </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
           <t>routes</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>$B$6</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4">
-        <f>CALIBRATIONREPORT.GET.OBSERVATIONS($B$16)</f>
-        <v/>
-      </c>
-    </row>
+      <c r="E22" s="6">
+        <f>$B$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24"/>
     <row r="25">
       <c r="D25" s="2" t="inlineStr">
@@ -8657,11 +9184,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>Fitted parameters</t>
-        </is>
-      </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
           <t>jacobian_mode</t>
@@ -8674,10 +9196,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4">
-        <f>CALIBRATIONREPORT.GET.PARAMETERS($B$16)</f>
-        <v/>
-      </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
           <t>difference_step</t>
@@ -8717,10 +9235,9 @@
           <t>geometry</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>$B$5</t>
-        </is>
+      <c r="E46" s="6">
+        <f>$B$5</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -8729,10 +9246,9 @@
           <t>market</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>$B$7</t>
-        </is>
+      <c r="E47" s="6">
+        <f>$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -8741,10 +9257,9 @@
           <t>valuation</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>$B$9</t>
-        </is>
+      <c r="E48" s="6">
+        <f>$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -8753,10 +9268,9 @@
           <t>observations</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>$B$12</t>
-        </is>
+      <c r="E49" s="6">
+        <f>$B$12</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -8765,11 +9279,526 @@
           <t>solver</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>$B$10</t>
-        </is>
-      </c>
+      <c r="E50" s="6">
+        <f>$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>Observation report</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="8">
+        <f t="array" ref="A55:V68">CALIBRATIONREPORT.GET.OBSERVATIONS($B$16)</f>
+        <v/>
+      </c>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8" t="n"/>
+      <c r="K55" s="8" t="n"/>
+      <c r="L55" s="9" t="n"/>
+      <c r="M55" s="8" t="n"/>
+      <c r="N55" s="9" t="n"/>
+      <c r="O55" s="9" t="n"/>
+      <c r="P55" s="8" t="n"/>
+      <c r="Q55" s="8" t="n"/>
+      <c r="R55" s="8" t="n"/>
+      <c r="S55" s="8" t="n"/>
+      <c r="T55" s="8" t="n"/>
+      <c r="U55" s="8" t="n"/>
+      <c r="V55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n"/>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="10" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="10" t="n"/>
+      <c r="I56" s="10" t="n"/>
+      <c r="J56" s="10" t="n"/>
+      <c r="K56" s="10" t="n"/>
+      <c r="L56" s="11" t="n"/>
+      <c r="M56" s="10" t="n"/>
+      <c r="N56" s="11" t="n"/>
+      <c r="O56" s="11" t="n"/>
+      <c r="P56" s="10" t="n"/>
+      <c r="Q56" s="10" t="n"/>
+      <c r="R56" s="10" t="n"/>
+      <c r="S56" s="10" t="n"/>
+      <c r="T56" s="10" t="n"/>
+      <c r="U56" s="10" t="n"/>
+      <c r="V56" s="10" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="n"/>
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="10" t="n"/>
+      <c r="D57" s="10" t="n"/>
+      <c r="E57" s="10" t="n"/>
+      <c r="F57" s="10" t="n"/>
+      <c r="G57" s="10" t="n"/>
+      <c r="H57" s="10" t="n"/>
+      <c r="I57" s="10" t="n"/>
+      <c r="J57" s="10" t="n"/>
+      <c r="K57" s="10" t="n"/>
+      <c r="L57" s="11" t="n"/>
+      <c r="M57" s="10" t="n"/>
+      <c r="N57" s="11" t="n"/>
+      <c r="O57" s="11" t="n"/>
+      <c r="P57" s="10" t="n"/>
+      <c r="Q57" s="10" t="n"/>
+      <c r="R57" s="10" t="n"/>
+      <c r="S57" s="10" t="n"/>
+      <c r="T57" s="10" t="n"/>
+      <c r="U57" s="10" t="n"/>
+      <c r="V57" s="10" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n"/>
+      <c r="B58" s="10" t="n"/>
+      <c r="C58" s="10" t="n"/>
+      <c r="D58" s="10" t="n"/>
+      <c r="E58" s="10" t="n"/>
+      <c r="F58" s="10" t="n"/>
+      <c r="G58" s="10" t="n"/>
+      <c r="H58" s="10" t="n"/>
+      <c r="I58" s="10" t="n"/>
+      <c r="J58" s="10" t="n"/>
+      <c r="K58" s="10" t="n"/>
+      <c r="L58" s="11" t="n"/>
+      <c r="M58" s="10" t="n"/>
+      <c r="N58" s="11" t="n"/>
+      <c r="O58" s="11" t="n"/>
+      <c r="P58" s="10" t="n"/>
+      <c r="Q58" s="10" t="n"/>
+      <c r="R58" s="10" t="n"/>
+      <c r="S58" s="10" t="n"/>
+      <c r="T58" s="10" t="n"/>
+      <c r="U58" s="10" t="n"/>
+      <c r="V58" s="10" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="n"/>
+      <c r="B59" s="10" t="n"/>
+      <c r="C59" s="10" t="n"/>
+      <c r="D59" s="10" t="n"/>
+      <c r="E59" s="10" t="n"/>
+      <c r="F59" s="10" t="n"/>
+      <c r="G59" s="10" t="n"/>
+      <c r="H59" s="10" t="n"/>
+      <c r="I59" s="10" t="n"/>
+      <c r="J59" s="10" t="n"/>
+      <c r="K59" s="10" t="n"/>
+      <c r="L59" s="11" t="n"/>
+      <c r="M59" s="10" t="n"/>
+      <c r="N59" s="11" t="n"/>
+      <c r="O59" s="11" t="n"/>
+      <c r="P59" s="10" t="n"/>
+      <c r="Q59" s="10" t="n"/>
+      <c r="R59" s="10" t="n"/>
+      <c r="S59" s="10" t="n"/>
+      <c r="T59" s="10" t="n"/>
+      <c r="U59" s="10" t="n"/>
+      <c r="V59" s="10" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="n"/>
+      <c r="B60" s="10" t="n"/>
+      <c r="C60" s="10" t="n"/>
+      <c r="D60" s="10" t="n"/>
+      <c r="E60" s="10" t="n"/>
+      <c r="F60" s="10" t="n"/>
+      <c r="G60" s="10" t="n"/>
+      <c r="H60" s="10" t="n"/>
+      <c r="I60" s="10" t="n"/>
+      <c r="J60" s="10" t="n"/>
+      <c r="K60" s="10" t="n"/>
+      <c r="L60" s="11" t="n"/>
+      <c r="M60" s="10" t="n"/>
+      <c r="N60" s="11" t="n"/>
+      <c r="O60" s="11" t="n"/>
+      <c r="P60" s="10" t="n"/>
+      <c r="Q60" s="10" t="n"/>
+      <c r="R60" s="10" t="n"/>
+      <c r="S60" s="10" t="n"/>
+      <c r="T60" s="10" t="n"/>
+      <c r="U60" s="10" t="n"/>
+      <c r="V60" s="10" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="n"/>
+      <c r="B61" s="10" t="n"/>
+      <c r="C61" s="10" t="n"/>
+      <c r="D61" s="10" t="n"/>
+      <c r="E61" s="10" t="n"/>
+      <c r="F61" s="10" t="n"/>
+      <c r="G61" s="10" t="n"/>
+      <c r="H61" s="10" t="n"/>
+      <c r="I61" s="10" t="n"/>
+      <c r="J61" s="10" t="n"/>
+      <c r="K61" s="10" t="n"/>
+      <c r="L61" s="11" t="n"/>
+      <c r="M61" s="10" t="n"/>
+      <c r="N61" s="11" t="n"/>
+      <c r="O61" s="11" t="n"/>
+      <c r="P61" s="10" t="n"/>
+      <c r="Q61" s="10" t="n"/>
+      <c r="R61" s="10" t="n"/>
+      <c r="S61" s="10" t="n"/>
+      <c r="T61" s="10" t="n"/>
+      <c r="U61" s="10" t="n"/>
+      <c r="V61" s="10" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="n"/>
+      <c r="B62" s="10" t="n"/>
+      <c r="C62" s="10" t="n"/>
+      <c r="D62" s="10" t="n"/>
+      <c r="E62" s="10" t="n"/>
+      <c r="F62" s="10" t="n"/>
+      <c r="G62" s="10" t="n"/>
+      <c r="H62" s="10" t="n"/>
+      <c r="I62" s="10" t="n"/>
+      <c r="J62" s="10" t="n"/>
+      <c r="K62" s="10" t="n"/>
+      <c r="L62" s="11" t="n"/>
+      <c r="M62" s="10" t="n"/>
+      <c r="N62" s="11" t="n"/>
+      <c r="O62" s="11" t="n"/>
+      <c r="P62" s="10" t="n"/>
+      <c r="Q62" s="10" t="n"/>
+      <c r="R62" s="10" t="n"/>
+      <c r="S62" s="10" t="n"/>
+      <c r="T62" s="10" t="n"/>
+      <c r="U62" s="10" t="n"/>
+      <c r="V62" s="10" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="n"/>
+      <c r="B63" s="10" t="n"/>
+      <c r="C63" s="10" t="n"/>
+      <c r="D63" s="10" t="n"/>
+      <c r="E63" s="10" t="n"/>
+      <c r="F63" s="10" t="n"/>
+      <c r="G63" s="10" t="n"/>
+      <c r="H63" s="10" t="n"/>
+      <c r="I63" s="10" t="n"/>
+      <c r="J63" s="10" t="n"/>
+      <c r="K63" s="10" t="n"/>
+      <c r="L63" s="11" t="n"/>
+      <c r="M63" s="10" t="n"/>
+      <c r="N63" s="11" t="n"/>
+      <c r="O63" s="11" t="n"/>
+      <c r="P63" s="10" t="n"/>
+      <c r="Q63" s="10" t="n"/>
+      <c r="R63" s="10" t="n"/>
+      <c r="S63" s="10" t="n"/>
+      <c r="T63" s="10" t="n"/>
+      <c r="U63" s="10" t="n"/>
+      <c r="V63" s="10" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="n"/>
+      <c r="B64" s="10" t="n"/>
+      <c r="C64" s="10" t="n"/>
+      <c r="D64" s="10" t="n"/>
+      <c r="E64" s="10" t="n"/>
+      <c r="F64" s="10" t="n"/>
+      <c r="G64" s="10" t="n"/>
+      <c r="H64" s="10" t="n"/>
+      <c r="I64" s="10" t="n"/>
+      <c r="J64" s="10" t="n"/>
+      <c r="K64" s="10" t="n"/>
+      <c r="L64" s="11" t="n"/>
+      <c r="M64" s="10" t="n"/>
+      <c r="N64" s="11" t="n"/>
+      <c r="O64" s="11" t="n"/>
+      <c r="P64" s="10" t="n"/>
+      <c r="Q64" s="10" t="n"/>
+      <c r="R64" s="10" t="n"/>
+      <c r="S64" s="10" t="n"/>
+      <c r="T64" s="10" t="n"/>
+      <c r="U64" s="10" t="n"/>
+      <c r="V64" s="10" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="n"/>
+      <c r="B65" s="10" t="n"/>
+      <c r="C65" s="10" t="n"/>
+      <c r="D65" s="10" t="n"/>
+      <c r="E65" s="10" t="n"/>
+      <c r="F65" s="10" t="n"/>
+      <c r="G65" s="10" t="n"/>
+      <c r="H65" s="10" t="n"/>
+      <c r="I65" s="10" t="n"/>
+      <c r="J65" s="10" t="n"/>
+      <c r="K65" s="10" t="n"/>
+      <c r="L65" s="11" t="n"/>
+      <c r="M65" s="10" t="n"/>
+      <c r="N65" s="11" t="n"/>
+      <c r="O65" s="11" t="n"/>
+      <c r="P65" s="10" t="n"/>
+      <c r="Q65" s="10" t="n"/>
+      <c r="R65" s="10" t="n"/>
+      <c r="S65" s="10" t="n"/>
+      <c r="T65" s="10" t="n"/>
+      <c r="U65" s="10" t="n"/>
+      <c r="V65" s="10" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="n"/>
+      <c r="B66" s="10" t="n"/>
+      <c r="C66" s="10" t="n"/>
+      <c r="D66" s="10" t="n"/>
+      <c r="E66" s="10" t="n"/>
+      <c r="F66" s="10" t="n"/>
+      <c r="G66" s="10" t="n"/>
+      <c r="H66" s="10" t="n"/>
+      <c r="I66" s="10" t="n"/>
+      <c r="J66" s="10" t="n"/>
+      <c r="K66" s="10" t="n"/>
+      <c r="L66" s="11" t="n"/>
+      <c r="M66" s="10" t="n"/>
+      <c r="N66" s="11" t="n"/>
+      <c r="O66" s="11" t="n"/>
+      <c r="P66" s="10" t="n"/>
+      <c r="Q66" s="10" t="n"/>
+      <c r="R66" s="10" t="n"/>
+      <c r="S66" s="10" t="n"/>
+      <c r="T66" s="10" t="n"/>
+      <c r="U66" s="10" t="n"/>
+      <c r="V66" s="10" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="n"/>
+      <c r="B67" s="10" t="n"/>
+      <c r="C67" s="10" t="n"/>
+      <c r="D67" s="10" t="n"/>
+      <c r="E67" s="10" t="n"/>
+      <c r="F67" s="10" t="n"/>
+      <c r="G67" s="10" t="n"/>
+      <c r="H67" s="10" t="n"/>
+      <c r="I67" s="10" t="n"/>
+      <c r="J67" s="10" t="n"/>
+      <c r="K67" s="10" t="n"/>
+      <c r="L67" s="11" t="n"/>
+      <c r="M67" s="10" t="n"/>
+      <c r="N67" s="11" t="n"/>
+      <c r="O67" s="11" t="n"/>
+      <c r="P67" s="10" t="n"/>
+      <c r="Q67" s="10" t="n"/>
+      <c r="R67" s="10" t="n"/>
+      <c r="S67" s="10" t="n"/>
+      <c r="T67" s="10" t="n"/>
+      <c r="U67" s="10" t="n"/>
+      <c r="V67" s="10" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="n"/>
+      <c r="B68" s="10" t="n"/>
+      <c r="C68" s="10" t="n"/>
+      <c r="D68" s="10" t="n"/>
+      <c r="E68" s="10" t="n"/>
+      <c r="F68" s="10" t="n"/>
+      <c r="G68" s="10" t="n"/>
+      <c r="H68" s="10" t="n"/>
+      <c r="I68" s="10" t="n"/>
+      <c r="J68" s="10" t="n"/>
+      <c r="K68" s="10" t="n"/>
+      <c r="L68" s="11" t="n"/>
+      <c r="M68" s="10" t="n"/>
+      <c r="N68" s="11" t="n"/>
+      <c r="O68" s="11" t="n"/>
+      <c r="P68" s="10" t="n"/>
+      <c r="Q68" s="10" t="n"/>
+      <c r="R68" s="10" t="n"/>
+      <c r="S68" s="10" t="n"/>
+      <c r="T68" s="10" t="n"/>
+      <c r="U68" s="10" t="n"/>
+      <c r="V68" s="10" t="n"/>
+    </row>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>Fitted parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="32" customHeight="1">
+      <c r="A73" s="8">
+        <f t="array" ref="A73:I86">CALIBRATIONREPORT.GET.PARAMETERS($B$16)</f>
+        <v/>
+      </c>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="8" t="n"/>
+      <c r="D73" s="8" t="n"/>
+      <c r="E73" s="8" t="n"/>
+      <c r="F73" s="8" t="n"/>
+      <c r="G73" s="8" t="n"/>
+      <c r="H73" s="8" t="n"/>
+      <c r="I73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="n"/>
+      <c r="B74" s="10" t="n"/>
+      <c r="C74" s="10" t="n"/>
+      <c r="D74" s="10" t="n"/>
+      <c r="E74" s="10" t="n"/>
+      <c r="F74" s="10" t="n"/>
+      <c r="G74" s="10" t="n"/>
+      <c r="H74" s="10" t="n"/>
+      <c r="I74" s="10" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="n"/>
+      <c r="B75" s="10" t="n"/>
+      <c r="C75" s="10" t="n"/>
+      <c r="D75" s="10" t="n"/>
+      <c r="E75" s="10" t="n"/>
+      <c r="F75" s="10" t="n"/>
+      <c r="G75" s="10" t="n"/>
+      <c r="H75" s="10" t="n"/>
+      <c r="I75" s="10" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="n"/>
+      <c r="B76" s="10" t="n"/>
+      <c r="C76" s="10" t="n"/>
+      <c r="D76" s="10" t="n"/>
+      <c r="E76" s="10" t="n"/>
+      <c r="F76" s="10" t="n"/>
+      <c r="G76" s="10" t="n"/>
+      <c r="H76" s="10" t="n"/>
+      <c r="I76" s="10" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="n"/>
+      <c r="B77" s="10" t="n"/>
+      <c r="C77" s="10" t="n"/>
+      <c r="D77" s="10" t="n"/>
+      <c r="E77" s="10" t="n"/>
+      <c r="F77" s="10" t="n"/>
+      <c r="G77" s="10" t="n"/>
+      <c r="H77" s="10" t="n"/>
+      <c r="I77" s="10" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="n"/>
+      <c r="B78" s="10" t="n"/>
+      <c r="C78" s="10" t="n"/>
+      <c r="D78" s="10" t="n"/>
+      <c r="E78" s="10" t="n"/>
+      <c r="F78" s="10" t="n"/>
+      <c r="G78" s="10" t="n"/>
+      <c r="H78" s="10" t="n"/>
+      <c r="I78" s="10" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="n"/>
+      <c r="B79" s="10" t="n"/>
+      <c r="C79" s="10" t="n"/>
+      <c r="D79" s="10" t="n"/>
+      <c r="E79" s="10" t="n"/>
+      <c r="F79" s="10" t="n"/>
+      <c r="G79" s="10" t="n"/>
+      <c r="H79" s="10" t="n"/>
+      <c r="I79" s="10" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="n"/>
+      <c r="B80" s="10" t="n"/>
+      <c r="C80" s="10" t="n"/>
+      <c r="D80" s="10" t="n"/>
+      <c r="E80" s="10" t="n"/>
+      <c r="F80" s="10" t="n"/>
+      <c r="G80" s="10" t="n"/>
+      <c r="H80" s="10" t="n"/>
+      <c r="I80" s="10" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="n"/>
+      <c r="B81" s="10" t="n"/>
+      <c r="C81" s="10" t="n"/>
+      <c r="D81" s="10" t="n"/>
+      <c r="E81" s="10" t="n"/>
+      <c r="F81" s="10" t="n"/>
+      <c r="G81" s="10" t="n"/>
+      <c r="H81" s="10" t="n"/>
+      <c r="I81" s="10" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="n"/>
+      <c r="B82" s="10" t="n"/>
+      <c r="C82" s="10" t="n"/>
+      <c r="D82" s="10" t="n"/>
+      <c r="E82" s="10" t="n"/>
+      <c r="F82" s="10" t="n"/>
+      <c r="G82" s="10" t="n"/>
+      <c r="H82" s="10" t="n"/>
+      <c r="I82" s="10" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="n"/>
+      <c r="B83" s="10" t="n"/>
+      <c r="C83" s="10" t="n"/>
+      <c r="D83" s="10" t="n"/>
+      <c r="E83" s="10" t="n"/>
+      <c r="F83" s="10" t="n"/>
+      <c r="G83" s="10" t="n"/>
+      <c r="H83" s="10" t="n"/>
+      <c r="I83" s="10" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="n"/>
+      <c r="B84" s="10" t="n"/>
+      <c r="C84" s="10" t="n"/>
+      <c r="D84" s="10" t="n"/>
+      <c r="E84" s="10" t="n"/>
+      <c r="F84" s="10" t="n"/>
+      <c r="G84" s="10" t="n"/>
+      <c r="H84" s="10" t="n"/>
+      <c r="I84" s="10" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="n"/>
+      <c r="B85" s="10" t="n"/>
+      <c r="C85" s="10" t="n"/>
+      <c r="D85" s="10" t="n"/>
+      <c r="E85" s="10" t="n"/>
+      <c r="F85" s="10" t="n"/>
+      <c r="G85" s="10" t="n"/>
+      <c r="H85" s="10" t="n"/>
+      <c r="I85" s="10" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="n"/>
+      <c r="B86" s="10" t="n"/>
+      <c r="C86" s="10" t="n"/>
+      <c r="D86" s="10" t="n"/>
+      <c r="E86" s="10" t="n"/>
+      <c r="F86" s="10" t="n"/>
+      <c r="G86" s="10" t="n"/>
+      <c r="H86" s="10" t="n"/>
+      <c r="I86" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8782,17 +9811,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:V86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="67" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8817,7 +9860,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>CALIBRATIONDATES.NEW($H$5:$H$18)</f>
+        <f>CALIBRATIONDATES.NEW($L$5:$L$18)</f>
         <v/>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -8830,12 +9873,12 @@
           <t>value</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>knot_date</t>
         </is>
@@ -8848,7 +9891,7 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>CURVEINSTRUMENTGEOMETRY.NEW($D$4:$E$14)</f>
+        <f>CURVEINSTRUMENTGEOMETRY.NEW($D$5:$E$14)</f>
         <v/>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -8859,10 +9902,10 @@
       <c r="E5" s="7" t="n">
         <v>44562</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="K5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="L5" s="7" t="n">
         <v>44562</v>
       </c>
     </row>
@@ -8886,10 +9929,10 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="K6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="L6" s="7" t="n">
         <v>44635</v>
       </c>
     </row>
@@ -8900,7 +9943,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>CURVEINSTRUMENTMARKET.NEW($D$21:$E$22)</f>
+        <f>CURVEINSTRUMENTMARKET.NEW($D$22:$E$22)</f>
         <v/>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -8913,10 +9956,10 @@
           <t>ptirds</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="K7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="L7" s="7" t="n">
         <v>44727</v>
       </c>
     </row>
@@ -8935,15 +9978,14 @@
           <t>knot_dates</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>$B$4</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="n">
+      <c r="E8" s="6">
+        <f>$B$4</f>
+        <v/>
+      </c>
+      <c r="K8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="L8" s="7" t="n">
         <v>44825</v>
       </c>
     </row>
@@ -8954,7 +9996,7 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <f>SCRIPTVALUATIONSETTINGS.NEW("ptirds-valuation",$D$25:$E$26,$B$8)</f>
+        <f>SCRIPTVALUATIONSETTINGS.NEW("ptirds-valuation",$D$26:$E$26,$B$8)</f>
         <v/>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -8967,10 +10009,10 @@
           <t>LOG_DISCOUNT</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="K9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="L9" s="7" t="n">
         <v>44916</v>
       </c>
     </row>
@@ -8981,7 +10023,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>CURVEINSTRUMENTSOLVER.NEW($D$29:$E$35)</f>
+        <f>CURVEINSTRUMENTSOLVER.NEW($D$30:$E$35)</f>
         <v/>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -8994,10 +10036,10 @@
           <t>INPUT</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="K10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="L10" s="7" t="n">
         <v>45000</v>
       </c>
     </row>
@@ -9008,7 +10050,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>CURVEINSTRUMENTCALIBRATIONOPTIONS.NEW($D$38:$E$42)</f>
+        <f>CURVEINSTRUMENTCALIBRATIONOPTIONS.NEW($D$39:$E$42)</f>
         <v/>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -9021,10 +10063,10 @@
           <t>MIXED</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="L11" s="7" t="n">
         <v>45098</v>
       </c>
     </row>
@@ -9046,10 +10088,10 @@
       <c r="E12" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="K12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="L12" s="7" t="n">
         <v>45189</v>
       </c>
     </row>
@@ -9060,7 +10102,7 @@
         </is>
       </c>
       <c r="B13" s="4">
-        <f>CURVEINSTRUMENTCALIBRATIONSPEC.NEW($D$45:$E$50)</f>
+        <f>CURVEINSTRUMENTCALIBRATIONSPEC.NEW($D$46:$E$50)</f>
         <v/>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -9073,10 +10115,10 @@
           <t>OIS</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="K13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="L13" s="7" t="n">
         <v>45280</v>
       </c>
     </row>
@@ -9100,10 +10142,10 @@
           <t>ACT_365F</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="K14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="L14" s="7" t="n">
         <v>45366</v>
       </c>
     </row>
@@ -9117,10 +10159,10 @@
         <f>CALIBRATIONOUTCOME.GET.STATUS($B$14)</f>
         <v/>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="K15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="L15" s="7" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -9134,10 +10176,10 @@
         <f>CALIBRATIONOUTCOME.GET.REPORT($B$14)</f>
         <v/>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="K16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="H16" s="7" t="n">
+      <c r="L16" s="7" t="n">
         <v>46388</v>
       </c>
     </row>
@@ -9171,7 +10213,10 @@
           <t>tenor</t>
         </is>
       </c>
-      <c r="H17" s="7" t="n">
+      <c r="K17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L17" s="7" t="n">
         <v>47119</v>
       </c>
     </row>
@@ -9189,10 +10234,11 @@
           <t>OIS</t>
         </is>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="6" t="n"/>
+      <c r="K18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="L18" s="7" t="n">
         <v>48214</v>
       </c>
     </row>
@@ -9211,28 +10257,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Observation report</t>
-        </is>
-      </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
           <t>routes</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>$B$6</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4">
-        <f>CALIBRATIONREPORT.GET.OBSERVATIONS($B$16)</f>
-        <v/>
-      </c>
-    </row>
+      <c r="E22" s="6">
+        <f>$B$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24"/>
     <row r="25">
       <c r="D25" s="2" t="inlineStr">
@@ -9359,11 +10394,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>Fitted parameters</t>
-        </is>
-      </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
           <t>jacobian_mode</t>
@@ -9376,10 +10406,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4">
-        <f>CALIBRATIONREPORT.GET.PARAMETERS($B$16)</f>
-        <v/>
-      </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
           <t>difference_step</t>
@@ -9419,10 +10445,9 @@
           <t>geometry</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>$B$5</t>
-        </is>
+      <c r="E46" s="6">
+        <f>$B$5</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -9431,10 +10456,9 @@
           <t>market</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>$B$7</t>
-        </is>
+      <c r="E47" s="6">
+        <f>$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -9443,10 +10467,9 @@
           <t>valuation</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>$B$9</t>
-        </is>
+      <c r="E48" s="6">
+        <f>$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -9455,10 +10478,9 @@
           <t>observations</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>$B$12</t>
-        </is>
+      <c r="E49" s="6">
+        <f>$B$12</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -9467,11 +10489,526 @@
           <t>solver</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>$B$10</t>
-        </is>
-      </c>
+      <c r="E50" s="6">
+        <f>$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>Observation report</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="8">
+        <f t="array" ref="A55:V68">CALIBRATIONREPORT.GET.OBSERVATIONS($B$16)</f>
+        <v/>
+      </c>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8" t="n"/>
+      <c r="K55" s="8" t="n"/>
+      <c r="L55" s="9" t="n"/>
+      <c r="M55" s="8" t="n"/>
+      <c r="N55" s="9" t="n"/>
+      <c r="O55" s="9" t="n"/>
+      <c r="P55" s="8" t="n"/>
+      <c r="Q55" s="8" t="n"/>
+      <c r="R55" s="8" t="n"/>
+      <c r="S55" s="8" t="n"/>
+      <c r="T55" s="8" t="n"/>
+      <c r="U55" s="8" t="n"/>
+      <c r="V55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n"/>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="10" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="10" t="n"/>
+      <c r="I56" s="10" t="n"/>
+      <c r="J56" s="10" t="n"/>
+      <c r="K56" s="10" t="n"/>
+      <c r="L56" s="11" t="n"/>
+      <c r="M56" s="10" t="n"/>
+      <c r="N56" s="11" t="n"/>
+      <c r="O56" s="11" t="n"/>
+      <c r="P56" s="10" t="n"/>
+      <c r="Q56" s="10" t="n"/>
+      <c r="R56" s="10" t="n"/>
+      <c r="S56" s="10" t="n"/>
+      <c r="T56" s="10" t="n"/>
+      <c r="U56" s="10" t="n"/>
+      <c r="V56" s="10" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="n"/>
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="10" t="n"/>
+      <c r="D57" s="10" t="n"/>
+      <c r="E57" s="10" t="n"/>
+      <c r="F57" s="10" t="n"/>
+      <c r="G57" s="10" t="n"/>
+      <c r="H57" s="10" t="n"/>
+      <c r="I57" s="10" t="n"/>
+      <c r="J57" s="10" t="n"/>
+      <c r="K57" s="10" t="n"/>
+      <c r="L57" s="11" t="n"/>
+      <c r="M57" s="10" t="n"/>
+      <c r="N57" s="11" t="n"/>
+      <c r="O57" s="11" t="n"/>
+      <c r="P57" s="10" t="n"/>
+      <c r="Q57" s="10" t="n"/>
+      <c r="R57" s="10" t="n"/>
+      <c r="S57" s="10" t="n"/>
+      <c r="T57" s="10" t="n"/>
+      <c r="U57" s="10" t="n"/>
+      <c r="V57" s="10" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n"/>
+      <c r="B58" s="10" t="n"/>
+      <c r="C58" s="10" t="n"/>
+      <c r="D58" s="10" t="n"/>
+      <c r="E58" s="10" t="n"/>
+      <c r="F58" s="10" t="n"/>
+      <c r="G58" s="10" t="n"/>
+      <c r="H58" s="10" t="n"/>
+      <c r="I58" s="10" t="n"/>
+      <c r="J58" s="10" t="n"/>
+      <c r="K58" s="10" t="n"/>
+      <c r="L58" s="11" t="n"/>
+      <c r="M58" s="10" t="n"/>
+      <c r="N58" s="11" t="n"/>
+      <c r="O58" s="11" t="n"/>
+      <c r="P58" s="10" t="n"/>
+      <c r="Q58" s="10" t="n"/>
+      <c r="R58" s="10" t="n"/>
+      <c r="S58" s="10" t="n"/>
+      <c r="T58" s="10" t="n"/>
+      <c r="U58" s="10" t="n"/>
+      <c r="V58" s="10" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="n"/>
+      <c r="B59" s="10" t="n"/>
+      <c r="C59" s="10" t="n"/>
+      <c r="D59" s="10" t="n"/>
+      <c r="E59" s="10" t="n"/>
+      <c r="F59" s="10" t="n"/>
+      <c r="G59" s="10" t="n"/>
+      <c r="H59" s="10" t="n"/>
+      <c r="I59" s="10" t="n"/>
+      <c r="J59" s="10" t="n"/>
+      <c r="K59" s="10" t="n"/>
+      <c r="L59" s="11" t="n"/>
+      <c r="M59" s="10" t="n"/>
+      <c r="N59" s="11" t="n"/>
+      <c r="O59" s="11" t="n"/>
+      <c r="P59" s="10" t="n"/>
+      <c r="Q59" s="10" t="n"/>
+      <c r="R59" s="10" t="n"/>
+      <c r="S59" s="10" t="n"/>
+      <c r="T59" s="10" t="n"/>
+      <c r="U59" s="10" t="n"/>
+      <c r="V59" s="10" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="n"/>
+      <c r="B60" s="10" t="n"/>
+      <c r="C60" s="10" t="n"/>
+      <c r="D60" s="10" t="n"/>
+      <c r="E60" s="10" t="n"/>
+      <c r="F60" s="10" t="n"/>
+      <c r="G60" s="10" t="n"/>
+      <c r="H60" s="10" t="n"/>
+      <c r="I60" s="10" t="n"/>
+      <c r="J60" s="10" t="n"/>
+      <c r="K60" s="10" t="n"/>
+      <c r="L60" s="11" t="n"/>
+      <c r="M60" s="10" t="n"/>
+      <c r="N60" s="11" t="n"/>
+      <c r="O60" s="11" t="n"/>
+      <c r="P60" s="10" t="n"/>
+      <c r="Q60" s="10" t="n"/>
+      <c r="R60" s="10" t="n"/>
+      <c r="S60" s="10" t="n"/>
+      <c r="T60" s="10" t="n"/>
+      <c r="U60" s="10" t="n"/>
+      <c r="V60" s="10" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="n"/>
+      <c r="B61" s="10" t="n"/>
+      <c r="C61" s="10" t="n"/>
+      <c r="D61" s="10" t="n"/>
+      <c r="E61" s="10" t="n"/>
+      <c r="F61" s="10" t="n"/>
+      <c r="G61" s="10" t="n"/>
+      <c r="H61" s="10" t="n"/>
+      <c r="I61" s="10" t="n"/>
+      <c r="J61" s="10" t="n"/>
+      <c r="K61" s="10" t="n"/>
+      <c r="L61" s="11" t="n"/>
+      <c r="M61" s="10" t="n"/>
+      <c r="N61" s="11" t="n"/>
+      <c r="O61" s="11" t="n"/>
+      <c r="P61" s="10" t="n"/>
+      <c r="Q61" s="10" t="n"/>
+      <c r="R61" s="10" t="n"/>
+      <c r="S61" s="10" t="n"/>
+      <c r="T61" s="10" t="n"/>
+      <c r="U61" s="10" t="n"/>
+      <c r="V61" s="10" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="n"/>
+      <c r="B62" s="10" t="n"/>
+      <c r="C62" s="10" t="n"/>
+      <c r="D62" s="10" t="n"/>
+      <c r="E62" s="10" t="n"/>
+      <c r="F62" s="10" t="n"/>
+      <c r="G62" s="10" t="n"/>
+      <c r="H62" s="10" t="n"/>
+      <c r="I62" s="10" t="n"/>
+      <c r="J62" s="10" t="n"/>
+      <c r="K62" s="10" t="n"/>
+      <c r="L62" s="11" t="n"/>
+      <c r="M62" s="10" t="n"/>
+      <c r="N62" s="11" t="n"/>
+      <c r="O62" s="11" t="n"/>
+      <c r="P62" s="10" t="n"/>
+      <c r="Q62" s="10" t="n"/>
+      <c r="R62" s="10" t="n"/>
+      <c r="S62" s="10" t="n"/>
+      <c r="T62" s="10" t="n"/>
+      <c r="U62" s="10" t="n"/>
+      <c r="V62" s="10" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="n"/>
+      <c r="B63" s="10" t="n"/>
+      <c r="C63" s="10" t="n"/>
+      <c r="D63" s="10" t="n"/>
+      <c r="E63" s="10" t="n"/>
+      <c r="F63" s="10" t="n"/>
+      <c r="G63" s="10" t="n"/>
+      <c r="H63" s="10" t="n"/>
+      <c r="I63" s="10" t="n"/>
+      <c r="J63" s="10" t="n"/>
+      <c r="K63" s="10" t="n"/>
+      <c r="L63" s="11" t="n"/>
+      <c r="M63" s="10" t="n"/>
+      <c r="N63" s="11" t="n"/>
+      <c r="O63" s="11" t="n"/>
+      <c r="P63" s="10" t="n"/>
+      <c r="Q63" s="10" t="n"/>
+      <c r="R63" s="10" t="n"/>
+      <c r="S63" s="10" t="n"/>
+      <c r="T63" s="10" t="n"/>
+      <c r="U63" s="10" t="n"/>
+      <c r="V63" s="10" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="n"/>
+      <c r="B64" s="10" t="n"/>
+      <c r="C64" s="10" t="n"/>
+      <c r="D64" s="10" t="n"/>
+      <c r="E64" s="10" t="n"/>
+      <c r="F64" s="10" t="n"/>
+      <c r="G64" s="10" t="n"/>
+      <c r="H64" s="10" t="n"/>
+      <c r="I64" s="10" t="n"/>
+      <c r="J64" s="10" t="n"/>
+      <c r="K64" s="10" t="n"/>
+      <c r="L64" s="11" t="n"/>
+      <c r="M64" s="10" t="n"/>
+      <c r="N64" s="11" t="n"/>
+      <c r="O64" s="11" t="n"/>
+      <c r="P64" s="10" t="n"/>
+      <c r="Q64" s="10" t="n"/>
+      <c r="R64" s="10" t="n"/>
+      <c r="S64" s="10" t="n"/>
+      <c r="T64" s="10" t="n"/>
+      <c r="U64" s="10" t="n"/>
+      <c r="V64" s="10" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="n"/>
+      <c r="B65" s="10" t="n"/>
+      <c r="C65" s="10" t="n"/>
+      <c r="D65" s="10" t="n"/>
+      <c r="E65" s="10" t="n"/>
+      <c r="F65" s="10" t="n"/>
+      <c r="G65" s="10" t="n"/>
+      <c r="H65" s="10" t="n"/>
+      <c r="I65" s="10" t="n"/>
+      <c r="J65" s="10" t="n"/>
+      <c r="K65" s="10" t="n"/>
+      <c r="L65" s="11" t="n"/>
+      <c r="M65" s="10" t="n"/>
+      <c r="N65" s="11" t="n"/>
+      <c r="O65" s="11" t="n"/>
+      <c r="P65" s="10" t="n"/>
+      <c r="Q65" s="10" t="n"/>
+      <c r="R65" s="10" t="n"/>
+      <c r="S65" s="10" t="n"/>
+      <c r="T65" s="10" t="n"/>
+      <c r="U65" s="10" t="n"/>
+      <c r="V65" s="10" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="n"/>
+      <c r="B66" s="10" t="n"/>
+      <c r="C66" s="10" t="n"/>
+      <c r="D66" s="10" t="n"/>
+      <c r="E66" s="10" t="n"/>
+      <c r="F66" s="10" t="n"/>
+      <c r="G66" s="10" t="n"/>
+      <c r="H66" s="10" t="n"/>
+      <c r="I66" s="10" t="n"/>
+      <c r="J66" s="10" t="n"/>
+      <c r="K66" s="10" t="n"/>
+      <c r="L66" s="11" t="n"/>
+      <c r="M66" s="10" t="n"/>
+      <c r="N66" s="11" t="n"/>
+      <c r="O66" s="11" t="n"/>
+      <c r="P66" s="10" t="n"/>
+      <c r="Q66" s="10" t="n"/>
+      <c r="R66" s="10" t="n"/>
+      <c r="S66" s="10" t="n"/>
+      <c r="T66" s="10" t="n"/>
+      <c r="U66" s="10" t="n"/>
+      <c r="V66" s="10" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="n"/>
+      <c r="B67" s="10" t="n"/>
+      <c r="C67" s="10" t="n"/>
+      <c r="D67" s="10" t="n"/>
+      <c r="E67" s="10" t="n"/>
+      <c r="F67" s="10" t="n"/>
+      <c r="G67" s="10" t="n"/>
+      <c r="H67" s="10" t="n"/>
+      <c r="I67" s="10" t="n"/>
+      <c r="J67" s="10" t="n"/>
+      <c r="K67" s="10" t="n"/>
+      <c r="L67" s="11" t="n"/>
+      <c r="M67" s="10" t="n"/>
+      <c r="N67" s="11" t="n"/>
+      <c r="O67" s="11" t="n"/>
+      <c r="P67" s="10" t="n"/>
+      <c r="Q67" s="10" t="n"/>
+      <c r="R67" s="10" t="n"/>
+      <c r="S67" s="10" t="n"/>
+      <c r="T67" s="10" t="n"/>
+      <c r="U67" s="10" t="n"/>
+      <c r="V67" s="10" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="n"/>
+      <c r="B68" s="10" t="n"/>
+      <c r="C68" s="10" t="n"/>
+      <c r="D68" s="10" t="n"/>
+      <c r="E68" s="10" t="n"/>
+      <c r="F68" s="10" t="n"/>
+      <c r="G68" s="10" t="n"/>
+      <c r="H68" s="10" t="n"/>
+      <c r="I68" s="10" t="n"/>
+      <c r="J68" s="10" t="n"/>
+      <c r="K68" s="10" t="n"/>
+      <c r="L68" s="11" t="n"/>
+      <c r="M68" s="10" t="n"/>
+      <c r="N68" s="11" t="n"/>
+      <c r="O68" s="11" t="n"/>
+      <c r="P68" s="10" t="n"/>
+      <c r="Q68" s="10" t="n"/>
+      <c r="R68" s="10" t="n"/>
+      <c r="S68" s="10" t="n"/>
+      <c r="T68" s="10" t="n"/>
+      <c r="U68" s="10" t="n"/>
+      <c r="V68" s="10" t="n"/>
+    </row>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>Fitted parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="32" customHeight="1">
+      <c r="A73" s="8">
+        <f t="array" ref="A73:I86">CALIBRATIONREPORT.GET.PARAMETERS($B$16)</f>
+        <v/>
+      </c>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="8" t="n"/>
+      <c r="D73" s="8" t="n"/>
+      <c r="E73" s="8" t="n"/>
+      <c r="F73" s="8" t="n"/>
+      <c r="G73" s="8" t="n"/>
+      <c r="H73" s="8" t="n"/>
+      <c r="I73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="n"/>
+      <c r="B74" s="10" t="n"/>
+      <c r="C74" s="10" t="n"/>
+      <c r="D74" s="10" t="n"/>
+      <c r="E74" s="10" t="n"/>
+      <c r="F74" s="10" t="n"/>
+      <c r="G74" s="10" t="n"/>
+      <c r="H74" s="10" t="n"/>
+      <c r="I74" s="10" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="n"/>
+      <c r="B75" s="10" t="n"/>
+      <c r="C75" s="10" t="n"/>
+      <c r="D75" s="10" t="n"/>
+      <c r="E75" s="10" t="n"/>
+      <c r="F75" s="10" t="n"/>
+      <c r="G75" s="10" t="n"/>
+      <c r="H75" s="10" t="n"/>
+      <c r="I75" s="10" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="n"/>
+      <c r="B76" s="10" t="n"/>
+      <c r="C76" s="10" t="n"/>
+      <c r="D76" s="10" t="n"/>
+      <c r="E76" s="10" t="n"/>
+      <c r="F76" s="10" t="n"/>
+      <c r="G76" s="10" t="n"/>
+      <c r="H76" s="10" t="n"/>
+      <c r="I76" s="10" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="n"/>
+      <c r="B77" s="10" t="n"/>
+      <c r="C77" s="10" t="n"/>
+      <c r="D77" s="10" t="n"/>
+      <c r="E77" s="10" t="n"/>
+      <c r="F77" s="10" t="n"/>
+      <c r="G77" s="10" t="n"/>
+      <c r="H77" s="10" t="n"/>
+      <c r="I77" s="10" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="n"/>
+      <c r="B78" s="10" t="n"/>
+      <c r="C78" s="10" t="n"/>
+      <c r="D78" s="10" t="n"/>
+      <c r="E78" s="10" t="n"/>
+      <c r="F78" s="10" t="n"/>
+      <c r="G78" s="10" t="n"/>
+      <c r="H78" s="10" t="n"/>
+      <c r="I78" s="10" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="n"/>
+      <c r="B79" s="10" t="n"/>
+      <c r="C79" s="10" t="n"/>
+      <c r="D79" s="10" t="n"/>
+      <c r="E79" s="10" t="n"/>
+      <c r="F79" s="10" t="n"/>
+      <c r="G79" s="10" t="n"/>
+      <c r="H79" s="10" t="n"/>
+      <c r="I79" s="10" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="n"/>
+      <c r="B80" s="10" t="n"/>
+      <c r="C80" s="10" t="n"/>
+      <c r="D80" s="10" t="n"/>
+      <c r="E80" s="10" t="n"/>
+      <c r="F80" s="10" t="n"/>
+      <c r="G80" s="10" t="n"/>
+      <c r="H80" s="10" t="n"/>
+      <c r="I80" s="10" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="n"/>
+      <c r="B81" s="10" t="n"/>
+      <c r="C81" s="10" t="n"/>
+      <c r="D81" s="10" t="n"/>
+      <c r="E81" s="10" t="n"/>
+      <c r="F81" s="10" t="n"/>
+      <c r="G81" s="10" t="n"/>
+      <c r="H81" s="10" t="n"/>
+      <c r="I81" s="10" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="n"/>
+      <c r="B82" s="10" t="n"/>
+      <c r="C82" s="10" t="n"/>
+      <c r="D82" s="10" t="n"/>
+      <c r="E82" s="10" t="n"/>
+      <c r="F82" s="10" t="n"/>
+      <c r="G82" s="10" t="n"/>
+      <c r="H82" s="10" t="n"/>
+      <c r="I82" s="10" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="n"/>
+      <c r="B83" s="10" t="n"/>
+      <c r="C83" s="10" t="n"/>
+      <c r="D83" s="10" t="n"/>
+      <c r="E83" s="10" t="n"/>
+      <c r="F83" s="10" t="n"/>
+      <c r="G83" s="10" t="n"/>
+      <c r="H83" s="10" t="n"/>
+      <c r="I83" s="10" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="n"/>
+      <c r="B84" s="10" t="n"/>
+      <c r="C84" s="10" t="n"/>
+      <c r="D84" s="10" t="n"/>
+      <c r="E84" s="10" t="n"/>
+      <c r="F84" s="10" t="n"/>
+      <c r="G84" s="10" t="n"/>
+      <c r="H84" s="10" t="n"/>
+      <c r="I84" s="10" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="n"/>
+      <c r="B85" s="10" t="n"/>
+      <c r="C85" s="10" t="n"/>
+      <c r="D85" s="10" t="n"/>
+      <c r="E85" s="10" t="n"/>
+      <c r="F85" s="10" t="n"/>
+      <c r="G85" s="10" t="n"/>
+      <c r="H85" s="10" t="n"/>
+      <c r="I85" s="10" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="n"/>
+      <c r="B86" s="10" t="n"/>
+      <c r="C86" s="10" t="n"/>
+      <c r="D86" s="10" t="n"/>
+      <c r="E86" s="10" t="n"/>
+      <c r="F86" s="10" t="n"/>
+      <c r="G86" s="10" t="n"/>
+      <c r="H86" s="10" t="n"/>
+      <c r="I86" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9487,7 +11024,7 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="115" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -9512,44 +11049,44 @@
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>The Instruments sheet constructs every definition from dated DAL script source rows. No native swap or native-to-script import function is used.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>The three calibration sheets share the same 13 instruments, quotes and 14 knots. Only log_discount_scheme changes: LOG_LINEAR, LOG_CUBIC_NATURAL and MIXED.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>ACT/365F accruals are unadjusted; the fixing date is the accrual start. N=100 and each K equals the original instrument's decimal par quote.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>The solver uses EXACT, initial guess 0.05, smoothing weight 1, 200 evaluations, 20 restarts and fit_norm_tolerance 1e-8. AAD is selected explicitly.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Run INIT.GLOBALDATA(1), then recalculate the workbook. CALIBRATIONOUTCOME.GET.STATUS should return Succeeded on all three sheets.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Observation and parameter tables are spilled from the typed report. This file contains formulas, not cached results; generating it does not execute Excel.</t>
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Observation and parameter tables use reserved array ranges below the input tables. This file contains formulas, not cached results; generating it does not execute Excel.</t>
         </is>
       </c>
     </row>

</xml_diff>